<commit_message>
enlarged the sample size of the dataset used for bettter ssas cubes
</commit_message>
<xml_diff>
--- a/Airlines_Source.xlsx
+++ b/Airlines_Source.xlsx
@@ -461,41 +461,41 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>UA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Delta Air Lines Inc.</t>
+          <t>United Air Lines Inc.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Delta Air Lines Inc.: DL</t>
+          <t>United Air Lines Inc.: UA</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>19790</v>
+        <v>19977</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UA</t>
+          <t>DL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>United Air Lines Inc.</t>
+          <t>Delta Air Lines Inc.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>United Air Lines Inc.: UA</t>
+          <t>Delta Air Lines Inc.: DL</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>19977</v>
+        <v>19790</v>
       </c>
     </row>
   </sheetData>

</xml_diff>